<commit_message>
Live price refresh + sold position fixes
- price_updater.py: fetches live prices via direct Yahoo API (no yfinance rate limits)
- FX logic: ticker suffix determines price currency (.NE/.TO = CAD, else USD × FX rate)
- Fixes .ME → .NE ticker typos, adds .TO for TSX ETFs
- Sold positions: rows with sold_market_value/book_cost_sold correctly classified
  (fixes ASML and similar positions showing in active)
- Updated Excel with corrected RESP quantities, IBIT.NE, currency fixes
- Realized P&L verified: $50,136 CAD

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Personal\Financial Accounts Trading Etc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD2A594F-93C9-4930-9930-E30FC599A9A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5FFC3E9-9389-49EC-B7AC-9112FC5D16C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{F25C29D6-FEA4-406D-91FC-6CA024EBB7CF}"/>
   </bookViews>
@@ -435,7 +435,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="978" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="980" uniqueCount="123">
   <si>
     <t>TFSA</t>
   </si>
@@ -659,9 +659,6 @@
     <t>Mkt_Val_Curr</t>
   </si>
   <si>
-    <t>VDY</t>
-  </si>
-  <si>
     <t>Index</t>
   </si>
   <si>
@@ -669,9 +666,6 @@
   </si>
   <si>
     <t>BURU</t>
-  </si>
-  <si>
-    <t>IBIT</t>
   </si>
   <si>
     <t>META</t>
@@ -764,15 +758,6 @@
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t>MU.ME</t>
-  </si>
-  <si>
-    <t>AMZN.ME</t>
-  </si>
-  <si>
-    <t>MSFT.ME</t>
-  </si>
-  <si>
     <t>Par_TICK</t>
   </si>
   <si>
@@ -785,9 +770,6 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>HOOD.ME</t>
-  </si>
-  <si>
     <t>zCash</t>
   </si>
   <si>
@@ -798,6 +780,30 @@
   </si>
   <si>
     <t>EUV</t>
+  </si>
+  <si>
+    <t>VDY.TO</t>
+  </si>
+  <si>
+    <t>MSFT.NE</t>
+  </si>
+  <si>
+    <t>MU.NE</t>
+  </si>
+  <si>
+    <t>HOOD.NE</t>
+  </si>
+  <si>
+    <t>AMZN.NE</t>
+  </si>
+  <si>
+    <t>AVGO.NE</t>
+  </si>
+  <si>
+    <t>META.ME</t>
+  </si>
+  <si>
+    <t>IBIT.NE</t>
   </si>
 </sst>
 </file>
@@ -1529,7 +1535,7 @@
         <v>11</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="E3" s="9" t="s">
         <v>2</v>
@@ -1630,7 +1636,7 @@
         <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D4" t="str">
         <f>C4</f>
@@ -1652,7 +1658,7 @@
         <v>5</v>
       </c>
       <c r="J4" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L4" s="1">
         <v>0</v>
@@ -1716,7 +1722,7 @@
         <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D5" t="str">
         <f t="shared" ref="D5:D68" si="9">C5</f>
@@ -1738,7 +1744,7 @@
         <v>5</v>
       </c>
       <c r="J5" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L5" s="1">
         <v>0</v>
@@ -1803,7 +1809,7 @@
         <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D6" t="str">
         <f t="shared" si="9"/>
@@ -1898,7 +1904,7 @@
         <v>38</v>
       </c>
       <c r="C7" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D7" t="str">
         <f t="shared" si="9"/>
@@ -1993,7 +1999,7 @@
         <v>38</v>
       </c>
       <c r="C8" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D8" t="str">
         <f t="shared" si="9"/>
@@ -2015,7 +2021,7 @@
         <v>5</v>
       </c>
       <c r="J8" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L8" s="1"/>
       <c r="M8" s="1">
@@ -2077,7 +2083,7 @@
         <v>38</v>
       </c>
       <c r="C9" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D9" t="str">
         <f t="shared" si="9"/>
@@ -2099,7 +2105,7 @@
         <v>5</v>
       </c>
       <c r="J9" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L9" s="1">
         <v>0</v>
@@ -2163,7 +2169,7 @@
         <v>38</v>
       </c>
       <c r="C10" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D10" t="str">
         <f t="shared" si="9"/>
@@ -2185,7 +2191,7 @@
         <v>5</v>
       </c>
       <c r="J10" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L10" s="1"/>
       <c r="M10" s="27">
@@ -2247,10 +2253,10 @@
         <v>38</v>
       </c>
       <c r="C11" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="D11" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E11" t="s">
         <v>6</v>
@@ -2339,7 +2345,7 @@
         <v>38</v>
       </c>
       <c r="C12" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D12" t="str">
         <f t="shared" si="9"/>
@@ -2361,7 +2367,7 @@
         <v>5</v>
       </c>
       <c r="J12" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L12" s="1">
         <v>8004</v>
@@ -2425,7 +2431,7 @@
         <v>38</v>
       </c>
       <c r="C13" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D13" t="str">
         <f t="shared" si="9"/>
@@ -2447,7 +2453,7 @@
         <v>5</v>
       </c>
       <c r="J13" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L13" s="1"/>
       <c r="M13" s="1">
@@ -2510,11 +2516,10 @@
         <v>38</v>
       </c>
       <c r="C14" t="s">
-        <v>76</v>
-      </c>
-      <c r="D14" t="str">
-        <f t="shared" si="9"/>
-        <v>AVGO</v>
+        <v>120</v>
+      </c>
+      <c r="D14" t="s">
+        <v>75</v>
       </c>
       <c r="E14" t="s">
         <v>6</v>
@@ -2601,11 +2606,11 @@
         <v>38</v>
       </c>
       <c r="C15" t="s">
-        <v>78</v>
+        <v>122</v>
       </c>
       <c r="D15" t="str">
         <f t="shared" si="9"/>
-        <v>IBIT</v>
+        <v>IBIT.NE</v>
       </c>
       <c r="E15" t="s">
         <v>6</v>
@@ -2643,7 +2648,7 @@
         <v>38.089199999999998</v>
       </c>
       <c r="T15" s="1">
-        <v>520</v>
+        <v>847</v>
       </c>
       <c r="U15" s="1"/>
       <c r="V15" s="1"/>
@@ -2692,11 +2697,10 @@
         <v>38</v>
       </c>
       <c r="C16" t="s">
-        <v>79</v>
-      </c>
-      <c r="D16" t="str">
-        <f t="shared" si="9"/>
-        <v>META</v>
+        <v>121</v>
+      </c>
+      <c r="D16" t="s">
+        <v>77</v>
       </c>
       <c r="E16" t="s">
         <v>6</v>
@@ -2783,10 +2787,10 @@
         <v>38</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E17" t="s">
         <v>6</v>
@@ -2824,7 +2828,7 @@
         <v>19.353300000000001</v>
       </c>
       <c r="T17" s="1">
-        <v>580</v>
+        <v>2900</v>
       </c>
       <c r="U17" s="1"/>
       <c r="V17" s="1"/>
@@ -2873,7 +2877,7 @@
         <v>38</v>
       </c>
       <c r="C18" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D18" t="str">
         <f t="shared" si="9"/>
@@ -2964,7 +2968,7 @@
         <v>38</v>
       </c>
       <c r="C19" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D19" t="str">
         <f t="shared" si="9"/>
@@ -3055,7 +3059,7 @@
         <v>38</v>
       </c>
       <c r="C20" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D20" t="str">
         <f t="shared" si="9"/>
@@ -3077,7 +3081,7 @@
         <v>5</v>
       </c>
       <c r="J20" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="K20" s="2"/>
       <c r="L20" s="1">
@@ -3140,7 +3144,7 @@
         <v>38</v>
       </c>
       <c r="C21" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D21" t="str">
         <f t="shared" si="9"/>
@@ -3162,7 +3166,7 @@
         <v>5</v>
       </c>
       <c r="J21" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="K21" s="2"/>
       <c r="L21" s="1"/>
@@ -3223,10 +3227,10 @@
         <v>38</v>
       </c>
       <c r="C22" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D22" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E22" t="s">
         <v>6</v>
@@ -3317,7 +3321,7 @@
         <v>38</v>
       </c>
       <c r="C23" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D23" t="str">
         <f t="shared" si="9"/>
@@ -3412,7 +3416,7 @@
         <v>38</v>
       </c>
       <c r="C24" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D24" t="str">
         <f t="shared" si="9"/>
@@ -3508,7 +3512,7 @@
         <v>38</v>
       </c>
       <c r="C25" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D25" t="str">
         <f t="shared" si="9"/>
@@ -3530,7 +3534,7 @@
         <v>5</v>
       </c>
       <c r="J25" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="K25" s="2"/>
       <c r="L25" s="1">
@@ -3538,7 +3542,7 @@
       </c>
       <c r="M25" s="1"/>
       <c r="N25" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="O25" s="1">
         <f>L25+M25</f>
@@ -3596,7 +3600,7 @@
         <v>38</v>
       </c>
       <c r="C26" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D26" t="str">
         <f t="shared" si="9"/>
@@ -3618,7 +3622,7 @@
         <v>5</v>
       </c>
       <c r="J26" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L26" s="1">
         <v>0</v>
@@ -3680,7 +3684,7 @@
         <v>38</v>
       </c>
       <c r="C27" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D27" t="str">
         <f t="shared" si="9"/>
@@ -3777,7 +3781,7 @@
         <v>38</v>
       </c>
       <c r="C28" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D28" t="str">
         <f t="shared" si="9"/>
@@ -3868,7 +3872,7 @@
         <v>38</v>
       </c>
       <c r="C29" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D29" t="str">
         <f t="shared" si="9"/>
@@ -3955,7 +3959,7 @@
     </row>
     <row r="30" spans="2:37" x14ac:dyDescent="0.45">
       <c r="B30" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C30" t="s">
         <v>49</v>
@@ -4052,7 +4056,7 @@
         <v>38</v>
       </c>
       <c r="C31" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D31" t="str">
         <f>C31</f>
@@ -4146,7 +4150,7 @@
         <v>38</v>
       </c>
       <c r="C32" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D32" t="str">
         <f t="shared" si="9"/>
@@ -4168,7 +4172,7 @@
         <v>5</v>
       </c>
       <c r="J32" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L32" s="1">
         <v>44.15</v>
@@ -4230,7 +4234,7 @@
         <v>38</v>
       </c>
       <c r="C33" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D33" t="s">
         <v>48</v>
@@ -4322,11 +4326,11 @@
         <v>38</v>
       </c>
       <c r="C34" t="s">
-        <v>74</v>
+        <v>115</v>
       </c>
       <c r="D34" t="str">
         <f t="shared" si="9"/>
-        <v>VDY</v>
+        <v>VDY.TO</v>
       </c>
       <c r="E34" t="s">
         <v>6</v>
@@ -4341,7 +4345,7 @@
         <v>45</v>
       </c>
       <c r="I34" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L34" s="1"/>
       <c r="M34" s="1"/>
@@ -4412,7 +4416,7 @@
         <v>38</v>
       </c>
       <c r="C35" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D35" t="str">
         <f t="shared" ref="D35:D36" si="78">C35</f>
@@ -4434,7 +4438,7 @@
         <v>5</v>
       </c>
       <c r="J35" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L35" s="1"/>
       <c r="M35" s="1">
@@ -4496,7 +4500,7 @@
         <v>38</v>
       </c>
       <c r="C36" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="D36" t="str">
         <f t="shared" si="78"/>
@@ -4589,7 +4593,7 @@
         <v>38</v>
       </c>
       <c r="C37" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D37" t="str">
         <f t="shared" si="9"/>
@@ -4679,7 +4683,7 @@
         <v>38</v>
       </c>
       <c r="C38" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D38" t="str">
         <f t="shared" si="9"/>
@@ -4772,7 +4776,7 @@
         <v>38</v>
       </c>
       <c r="C39" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D39" t="str">
         <f t="shared" si="9"/>
@@ -4862,7 +4866,7 @@
         <v>38</v>
       </c>
       <c r="C40" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D40" t="str">
         <f t="shared" si="9"/>
@@ -5044,7 +5048,7 @@
         <v>38</v>
       </c>
       <c r="C42" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D42" t="str">
         <f t="shared" si="9"/>
@@ -5230,7 +5234,7 @@
         <v>38</v>
       </c>
       <c r="C44" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D44" t="str">
         <f t="shared" si="9"/>
@@ -5249,7 +5253,7 @@
         <v>1</v>
       </c>
       <c r="I44" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L44" s="1"/>
       <c r="M44" s="1"/>
@@ -5318,7 +5322,7 @@
         <v>38</v>
       </c>
       <c r="C45" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D45" t="str">
         <f t="shared" si="9"/>
@@ -5410,7 +5414,7 @@
         <v>38</v>
       </c>
       <c r="C46" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D46" t="str">
         <f t="shared" si="9"/>
@@ -5432,7 +5436,7 @@
         <v>5</v>
       </c>
       <c r="J46" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L46" s="1">
         <v>0</v>
@@ -5490,7 +5494,7 @@
         <v>38</v>
       </c>
       <c r="C47" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D47" t="str">
         <f t="shared" si="9"/>
@@ -5512,7 +5516,7 @@
         <v>5</v>
       </c>
       <c r="J47" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L47" s="1">
         <v>0</v>
@@ -5573,7 +5577,7 @@
         <v>38</v>
       </c>
       <c r="C48" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D48" t="str">
         <f t="shared" si="9"/>
@@ -5595,7 +5599,7 @@
         <v>5</v>
       </c>
       <c r="J48" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L48" s="1">
         <v>10</v>
@@ -5653,7 +5657,7 @@
         <v>38</v>
       </c>
       <c r="C49" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D49" t="str">
         <f t="shared" si="9"/>
@@ -5675,7 +5679,7 @@
         <v>5</v>
       </c>
       <c r="J49" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L49" s="1">
         <v>0</v>
@@ -5735,7 +5739,7 @@
         <v>38</v>
       </c>
       <c r="C50" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D50" t="str">
         <f t="shared" si="9"/>
@@ -5757,7 +5761,7 @@
         <v>5</v>
       </c>
       <c r="J50" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L50" s="1">
         <v>0</v>
@@ -5817,7 +5821,7 @@
         <v>38</v>
       </c>
       <c r="C51" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D51" t="str">
         <f t="shared" si="9"/>
@@ -5839,7 +5843,7 @@
         <v>5</v>
       </c>
       <c r="J51" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L51" s="1"/>
       <c r="M51" s="1">
@@ -5897,7 +5901,7 @@
         <v>38</v>
       </c>
       <c r="C52" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D52" t="str">
         <f t="shared" si="9"/>
@@ -5919,7 +5923,7 @@
         <v>5</v>
       </c>
       <c r="J52" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L52" s="1">
         <v>57.58</v>
@@ -5977,7 +5981,7 @@
         <v>38</v>
       </c>
       <c r="C53" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D53" t="str">
         <f t="shared" si="9"/>
@@ -5999,7 +6003,7 @@
         <v>5</v>
       </c>
       <c r="J53" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L53" s="1"/>
       <c r="M53" s="1">
@@ -6057,7 +6061,7 @@
         <v>38</v>
       </c>
       <c r="C54" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D54" t="str">
         <f t="shared" si="9"/>
@@ -6079,7 +6083,7 @@
         <v>5</v>
       </c>
       <c r="J54" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L54" s="1">
         <v>0</v>
@@ -6139,7 +6143,7 @@
         <v>38</v>
       </c>
       <c r="C55" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D55" t="str">
         <f t="shared" si="9"/>
@@ -6161,7 +6165,7 @@
         <v>5</v>
       </c>
       <c r="J55" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L55" s="1"/>
       <c r="M55" s="1"/>
@@ -6217,7 +6221,7 @@
         <v>38</v>
       </c>
       <c r="C56" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D56" t="str">
         <f t="shared" si="9"/>
@@ -6239,7 +6243,7 @@
         <v>5</v>
       </c>
       <c r="J56" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L56" s="1">
         <v>0</v>
@@ -6297,7 +6301,7 @@
         <v>38</v>
       </c>
       <c r="C57" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D57" t="str">
         <f t="shared" si="9"/>
@@ -6319,7 +6323,7 @@
         <v>5</v>
       </c>
       <c r="J57" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L57" s="1">
         <v>119.38</v>
@@ -6377,7 +6381,7 @@
         <v>38</v>
       </c>
       <c r="C58" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D58" t="str">
         <f t="shared" si="9"/>
@@ -6464,7 +6468,7 @@
         <v>38</v>
       </c>
       <c r="C59" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="D59" t="str">
         <f t="shared" ref="D59" si="125">C59</f>
@@ -6554,7 +6558,7 @@
         <v>38</v>
       </c>
       <c r="C60" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="D60" t="str">
         <f t="shared" ref="D60" si="127">C60</f>
@@ -6644,7 +6648,7 @@
         <v>38</v>
       </c>
       <c r="C61" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D61" t="str">
         <f t="shared" si="9"/>
@@ -6734,7 +6738,7 @@
         <v>38</v>
       </c>
       <c r="C62" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D62" t="str">
         <f t="shared" si="9"/>
@@ -6821,7 +6825,7 @@
         <v>38</v>
       </c>
       <c r="C63" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="D63" t="str">
         <f t="shared" ref="D63" si="129">C63</f>
@@ -6911,7 +6915,7 @@
         <v>38</v>
       </c>
       <c r="C64" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D64" t="str">
         <f t="shared" si="9"/>
@@ -7001,7 +7005,7 @@
         <v>38</v>
       </c>
       <c r="C65" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D65" t="str">
         <f t="shared" si="9"/>
@@ -7023,7 +7027,7 @@
         <v>5</v>
       </c>
       <c r="J65" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L65" s="1">
         <v>0</v>
@@ -7081,10 +7085,10 @@
         <v>38</v>
       </c>
       <c r="C66" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="D66" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E66" t="s">
         <v>7</v>
@@ -7169,7 +7173,7 @@
         <v>38</v>
       </c>
       <c r="C67" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D67" t="str">
         <f t="shared" si="9"/>
@@ -7191,7 +7195,7 @@
         <v>5</v>
       </c>
       <c r="J67" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L67" s="1">
         <v>0</v>
@@ -7249,7 +7253,7 @@
         <v>38</v>
       </c>
       <c r="C68" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D68" t="str">
         <f t="shared" si="9"/>
@@ -7337,7 +7341,7 @@
         <v>38</v>
       </c>
       <c r="C69" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="D69" t="str">
         <f t="shared" ref="D69" si="158">C69</f>
@@ -7428,7 +7432,7 @@
         <v>38</v>
       </c>
       <c r="C70" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D70" t="str">
         <f t="shared" ref="D70:D81" si="160">C70</f>
@@ -7515,7 +7519,7 @@
         <v>38</v>
       </c>
       <c r="C71" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D71" t="str">
         <f t="shared" si="160"/>
@@ -7602,7 +7606,7 @@
         <v>38</v>
       </c>
       <c r="C72" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D72" t="str">
         <f t="shared" si="160"/>
@@ -7692,7 +7696,7 @@
         <v>38</v>
       </c>
       <c r="C73" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D73" t="str">
         <f t="shared" si="160"/>
@@ -7780,7 +7784,7 @@
         <v>38</v>
       </c>
       <c r="C74" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D74" t="str">
         <f t="shared" si="160"/>
@@ -7802,7 +7806,7 @@
         <v>5</v>
       </c>
       <c r="J74" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L74" s="1"/>
       <c r="M74" s="1"/>
@@ -7858,7 +7862,7 @@
         <v>38</v>
       </c>
       <c r="C75" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D75" t="str">
         <f t="shared" si="160"/>
@@ -7880,7 +7884,7 @@
         <v>5</v>
       </c>
       <c r="J75" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="L75" s="1">
         <v>249.72</v>
@@ -7942,7 +7946,7 @@
         <v>38</v>
       </c>
       <c r="C76" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D76" t="str">
         <f t="shared" si="160"/>
@@ -8030,7 +8034,7 @@
         <v>38</v>
       </c>
       <c r="C77" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D77" t="str">
         <f t="shared" si="160"/>
@@ -8117,7 +8121,7 @@
         <v>38</v>
       </c>
       <c r="C78" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D78" t="str">
         <f t="shared" si="160"/>
@@ -8207,7 +8211,7 @@
         <v>38</v>
       </c>
       <c r="C79" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D79" t="str">
         <f t="shared" si="160"/>
@@ -8226,7 +8230,7 @@
         <v>1</v>
       </c>
       <c r="I79" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J79" s="2">
         <v>45982</v>
@@ -8387,7 +8391,7 @@
         <v>38</v>
       </c>
       <c r="C81" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D81" t="str">
         <f t="shared" si="160"/>
@@ -8406,7 +8410,7 @@
         <v>1</v>
       </c>
       <c r="I81" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L81" s="1"/>
       <c r="M81" s="1"/>
@@ -8589,7 +8593,7 @@
         <v>38</v>
       </c>
       <c r="C89" s="8" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D89" s="8" t="str">
         <f>C89</f>
@@ -8695,7 +8699,7 @@
         <v>38</v>
       </c>
       <c r="C90" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D90" s="8" t="str">
         <f t="shared" ref="D90:D95" si="201">C90</f>
@@ -8799,7 +8803,7 @@
         <v>38</v>
       </c>
       <c r="C91" s="8" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D91" s="8" t="str">
         <f t="shared" si="201"/>
@@ -8908,7 +8912,7 @@
         <v>38</v>
       </c>
       <c r="C92" s="8" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D92" s="8" t="str">
         <f t="shared" si="201"/>
@@ -8927,7 +8931,7 @@
         <v>45</v>
       </c>
       <c r="I92" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K92" s="16">
         <v>46162</v>
@@ -8935,7 +8939,7 @@
       <c r="L92" s="17"/>
       <c r="M92" s="17"/>
       <c r="N92" s="17" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="O92" s="17">
         <f>L92+M92</f>
@@ -9014,7 +9018,7 @@
         <v>38</v>
       </c>
       <c r="C93" s="8" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D93" s="8" t="str">
         <f t="shared" si="201"/>
@@ -9033,7 +9037,7 @@
         <v>45</v>
       </c>
       <c r="I93" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K93" s="16">
         <v>46162</v>
@@ -9118,7 +9122,7 @@
         <v>38</v>
       </c>
       <c r="C94" s="8" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D94" s="8" t="str">
         <f t="shared" si="201"/>
@@ -9221,7 +9225,7 @@
         <v>38</v>
       </c>
       <c r="C95" s="8" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D95" s="8" t="str">
         <f t="shared" si="201"/>
@@ -9324,10 +9328,10 @@
         <v>38</v>
       </c>
       <c r="C96" s="8" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="D96" s="8" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E96" s="8" t="s">
         <v>6</v>
@@ -9530,7 +9534,7 @@
         <v>38</v>
       </c>
       <c r="C98" s="8" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E98" s="8" t="s">
         <v>6</v>
@@ -9633,7 +9637,7 @@
         <v>38</v>
       </c>
       <c r="C99" s="8" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E99" s="8" t="s">
         <v>7</v>
@@ -9735,7 +9739,7 @@
         <v>38</v>
       </c>
       <c r="C100" s="8" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E100" s="8" t="s">
         <v>6</v>
@@ -9830,7 +9834,7 @@
         <v>38</v>
       </c>
       <c r="C101" s="8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="E101" s="8" t="s">
         <v>6</v>
@@ -9927,7 +9931,7 @@
         <v>38</v>
       </c>
       <c r="C102" s="8" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E102" s="8" t="s">
         <v>6</v>
@@ -10121,7 +10125,7 @@
         <v>38</v>
       </c>
       <c r="C104" s="8" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E104" s="8" t="s">
         <v>6</v>
@@ -10136,7 +10140,7 @@
         <v>45</v>
       </c>
       <c r="I104" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K104" s="16">
         <v>46013</v>
@@ -10218,7 +10222,7 @@
         <v>38</v>
       </c>
       <c r="C105" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E105" s="8" t="s">
         <v>7</v>

</xml_diff>